<commit_message>
Update manual_references.xlsx with new data
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hamidrezabehbood/Documents/GitHub/FReD-data/cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103F3E61-A99E-BD4F-8763-5166EDA9D16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CCF5C8-837C-CD4F-B1CA-2BC239980651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="680" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="838">
   <si>
     <t>key</t>
   </si>
@@ -4970,6 +4970,27 @@
   </si>
   <si>
     <t>Article 13</t>
+  </si>
+  <si>
+    <t>10.1016/j.im.2015.06.009</t>
+  </si>
+  <si>
+    <t>Hsu, P.-F., Yen, H. R., &amp; Chung, J.-C. (2015). Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality. Information &amp; Management, 52(8), 925–942. https://doi.org/10.1016/j.im.2015.06.009</t>
+  </si>
+  <si>
+    <t>@article{Hsu2015ERP, author={Pei-Fang Hsu and HsiuJu Rebecca Yen and Jung-Ching Chung}, title={Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality}, journal={Information &amp; Management}, year={2015}, volume={52}, number={8}, pages={925--942}, doi={10.1016/j.im.2015.06.009} }</t>
+  </si>
+  <si>
+    <t>Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality</t>
+  </si>
+  <si>
+    <t>Hsu, Pei-Fang; Yen, HsiuJu Rebecca; Chung, Jung-Ching</t>
+  </si>
+  <si>
+    <t>Information &amp; Management</t>
+  </si>
+  <si>
+    <t>925-942</t>
   </si>
 </sst>
 </file>
@@ -5322,7 +5343,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J276"/>
+  <dimension ref="A1:J277"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -8862,6 +8883,38 @@
         <v>830</v>
       </c>
     </row>
+    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A277" t="s">
+        <v>831</v>
+      </c>
+      <c r="B277" t="s">
+        <v>832</v>
+      </c>
+      <c r="C277" t="s">
+        <v>833</v>
+      </c>
+      <c r="D277" t="s">
+        <v>834</v>
+      </c>
+      <c r="E277" t="s">
+        <v>835</v>
+      </c>
+      <c r="F277" t="s">
+        <v>836</v>
+      </c>
+      <c r="G277">
+        <v>2015</v>
+      </c>
+      <c r="H277">
+        <v>52</v>
+      </c>
+      <c r="I277">
+        <v>8</v>
+      </c>
+      <c r="J277" t="s">
+        <v>837</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update manual_references.xlsx with latest data
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hamidrezabehbood/Documents/GitHub/FReD-data/cache/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamid\Documents\GitHub\FReD-data\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CCF5C8-837C-CD4F-B1CA-2BC239980651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9CCA66-2D39-443F-90C4-180339AB495A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4300" yWindow="680" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="841">
   <si>
     <t>key</t>
   </si>
@@ -4992,12 +4992,21 @@
   <si>
     <t>925-942</t>
   </si>
+  <si>
+    <t>https://aisel.aisnet.org/trr/vol7/iss1/3</t>
+  </si>
+  <si>
+    <t>Kumar, M., &amp; Leroy, G. (2021). Factors Affecting Compliance with Alerts in the Context of Healthcare-related Emergencies. AIS Transactions on Replication Research, 7, Article 3. https://doi.org/10.17705/1atrr.00068</t>
+  </si>
+  <si>
+    <t>@article{kumar2021factors, title = {Factors Affecting Compliance with Alerts in the Context of Healthcare-related Emergencies}, author = {Kumar, Manasvi and Leroy, Gondy}, journal = {AIS Transactions on Replication Research}, year = {2021}, volume = {7}, number = {1}, note = {Article 3}, doi = {10.17705/1atrr.00068}, url = {https://aisel.aisnet.org/trr/vol7/iss1/3} }</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5009,6 +5018,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5034,11 +5050,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5343,10 +5360,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J277"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:SF278"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5378,7 +5395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -5389,7 +5406,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -5400,7 +5417,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -5411,7 +5428,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -5422,7 +5439,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -5433,7 +5450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -5444,7 +5461,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -5455,7 +5472,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -5466,7 +5483,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -5477,7 +5494,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -5488,7 +5505,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -5499,7 +5516,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -5510,7 +5527,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -5521,7 +5538,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>49</v>
       </c>
@@ -5532,7 +5549,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -5543,7 +5560,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -5554,7 +5571,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>58</v>
       </c>
@@ -5565,7 +5582,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -5576,7 +5593,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -5587,7 +5604,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>67</v>
       </c>
@@ -5598,7 +5615,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -5609,7 +5626,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -5620,7 +5637,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -5631,7 +5648,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -5642,7 +5659,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -5650,7 +5667,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>84</v>
       </c>
@@ -5661,7 +5678,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>87</v>
       </c>
@@ -5672,7 +5689,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>90</v>
       </c>
@@ -5683,7 +5700,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>93</v>
       </c>
@@ -5694,7 +5711,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>96</v>
       </c>
@@ -5705,7 +5722,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>99</v>
       </c>
@@ -5716,7 +5733,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>102</v>
       </c>
@@ -5727,7 +5744,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -5738,7 +5755,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>108</v>
       </c>
@@ -5749,7 +5766,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>111</v>
       </c>
@@ -5760,7 +5777,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>114</v>
       </c>
@@ -5771,7 +5788,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>117</v>
       </c>
@@ -5782,7 +5799,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>120</v>
       </c>
@@ -5793,7 +5810,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>123</v>
       </c>
@@ -5804,7 +5821,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>126</v>
       </c>
@@ -5815,7 +5832,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>129</v>
       </c>
@@ -5826,7 +5843,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>129</v>
       </c>
@@ -5837,7 +5854,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -5848,7 +5865,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>129</v>
       </c>
@@ -5859,7 +5876,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>132</v>
       </c>
@@ -5870,7 +5887,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>135</v>
       </c>
@@ -5881,7 +5898,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>135</v>
       </c>
@@ -5892,7 +5909,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -5903,7 +5920,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>138</v>
       </c>
@@ -5914,7 +5931,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>138</v>
       </c>
@@ -5925,7 +5942,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>138</v>
       </c>
@@ -5936,7 +5953,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>141</v>
       </c>
@@ -5947,7 +5964,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>144</v>
       </c>
@@ -5958,7 +5975,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>144</v>
       </c>
@@ -5969,7 +5986,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>144</v>
       </c>
@@ -5980,7 +5997,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>147</v>
       </c>
@@ -5991,7 +6008,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>147</v>
       </c>
@@ -6002,7 +6019,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>147</v>
       </c>
@@ -6013,7 +6030,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>147</v>
       </c>
@@ -6024,7 +6041,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>150</v>
       </c>
@@ -6035,7 +6052,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>153</v>
       </c>
@@ -6046,7 +6063,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>153</v>
       </c>
@@ -6057,7 +6074,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>156</v>
       </c>
@@ -6068,7 +6085,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>156</v>
       </c>
@@ -6079,7 +6096,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>156</v>
       </c>
@@ -6090,7 +6107,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>159</v>
       </c>
@@ -6101,7 +6118,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>159</v>
       </c>
@@ -6112,7 +6129,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>159</v>
       </c>
@@ -6123,7 +6140,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>162</v>
       </c>
@@ -6134,7 +6151,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>162</v>
       </c>
@@ -6145,7 +6162,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>162</v>
       </c>
@@ -6156,7 +6173,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>165</v>
       </c>
@@ -6167,7 +6184,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>168</v>
       </c>
@@ -6178,7 +6195,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>168</v>
       </c>
@@ -6189,7 +6206,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>171</v>
       </c>
@@ -6200,7 +6217,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>171</v>
       </c>
@@ -6211,7 +6228,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>174</v>
       </c>
@@ -6222,7 +6239,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>174</v>
       </c>
@@ -6233,7 +6250,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>174</v>
       </c>
@@ -6244,7 +6261,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>177</v>
       </c>
@@ -6255,7 +6272,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>177</v>
       </c>
@@ -6266,7 +6283,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>177</v>
       </c>
@@ -6277,7 +6294,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -6288,7 +6305,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>183</v>
       </c>
@@ -6299,7 +6316,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>186</v>
       </c>
@@ -6310,7 +6327,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>186</v>
       </c>
@@ -6321,7 +6338,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>189</v>
       </c>
@@ -6332,7 +6349,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>192</v>
       </c>
@@ -6343,7 +6360,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>195</v>
       </c>
@@ -6354,7 +6371,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>198</v>
       </c>
@@ -6365,7 +6382,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>201</v>
       </c>
@@ -6376,7 +6393,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>201</v>
       </c>
@@ -6387,7 +6404,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>201</v>
       </c>
@@ -6398,7 +6415,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>201</v>
       </c>
@@ -6409,7 +6426,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>201</v>
       </c>
@@ -6420,7 +6437,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>201</v>
       </c>
@@ -6431,7 +6448,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>201</v>
       </c>
@@ -6442,7 +6459,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>201</v>
       </c>
@@ -6453,7 +6470,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>204</v>
       </c>
@@ -6464,7 +6481,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>207</v>
       </c>
@@ -6475,7 +6492,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>207</v>
       </c>
@@ -6486,7 +6503,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>210</v>
       </c>
@@ -6497,7 +6514,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>213</v>
       </c>
@@ -6508,7 +6525,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>216</v>
       </c>
@@ -6519,7 +6536,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>219</v>
       </c>
@@ -6530,7 +6547,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>219</v>
       </c>
@@ -6541,7 +6558,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>219</v>
       </c>
@@ -6552,7 +6569,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>219</v>
       </c>
@@ -6563,7 +6580,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>222</v>
       </c>
@@ -6574,7 +6591,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>225</v>
       </c>
@@ -6585,7 +6602,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>228</v>
       </c>
@@ -6596,7 +6613,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>231</v>
       </c>
@@ -6607,7 +6624,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>234</v>
       </c>
@@ -6618,7 +6635,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>237</v>
       </c>
@@ -6629,7 +6646,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>240</v>
       </c>
@@ -6640,7 +6657,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>243</v>
       </c>
@@ -6651,7 +6668,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>246</v>
       </c>
@@ -6662,7 +6679,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>249</v>
       </c>
@@ -6673,7 +6690,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>252</v>
       </c>
@@ -6684,7 +6701,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>255</v>
       </c>
@@ -6695,7 +6712,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>258</v>
       </c>
@@ -6706,7 +6723,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>261</v>
       </c>
@@ -6717,7 +6734,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>264</v>
       </c>
@@ -6728,7 +6745,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>267</v>
       </c>
@@ -6739,7 +6756,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>270</v>
       </c>
@@ -6750,7 +6767,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>273</v>
       </c>
@@ -6761,7 +6778,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>276</v>
       </c>
@@ -6772,7 +6789,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>279</v>
       </c>
@@ -6783,7 +6800,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>282</v>
       </c>
@@ -6794,7 +6811,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>285</v>
       </c>
@@ -6805,7 +6822,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>288</v>
       </c>
@@ -6816,7 +6833,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>291</v>
       </c>
@@ -6827,7 +6844,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>294</v>
       </c>
@@ -6838,7 +6855,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>297</v>
       </c>
@@ -6849,7 +6866,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>300</v>
       </c>
@@ -6860,7 +6877,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>303</v>
       </c>
@@ -6871,7 +6888,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>306</v>
       </c>
@@ -6882,7 +6899,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>309</v>
       </c>
@@ -6893,7 +6910,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>312</v>
       </c>
@@ -6904,7 +6921,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>315</v>
       </c>
@@ -6915,7 +6932,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>318</v>
       </c>
@@ -6926,7 +6943,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>321</v>
       </c>
@@ -6937,7 +6954,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>324</v>
       </c>
@@ -6948,7 +6965,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>327</v>
       </c>
@@ -6959,7 +6976,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>330</v>
       </c>
@@ -6970,7 +6987,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>333</v>
       </c>
@@ -6981,7 +6998,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>336</v>
       </c>
@@ -6992,7 +7009,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>339</v>
       </c>
@@ -7003,7 +7020,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>342</v>
       </c>
@@ -7014,7 +7031,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>345</v>
       </c>
@@ -7025,7 +7042,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>348</v>
       </c>
@@ -7036,7 +7053,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>351</v>
       </c>
@@ -7047,7 +7064,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>354</v>
       </c>
@@ -7058,7 +7075,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>357</v>
       </c>
@@ -7069,7 +7086,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>360</v>
       </c>
@@ -7080,7 +7097,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>363</v>
       </c>
@@ -7091,7 +7108,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>366</v>
       </c>
@@ -7102,7 +7119,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>369</v>
       </c>
@@ -7113,7 +7130,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>372</v>
       </c>
@@ -7124,7 +7141,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>375</v>
       </c>
@@ -7135,7 +7152,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>378</v>
       </c>
@@ -7146,7 +7163,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>381</v>
       </c>
@@ -7157,7 +7174,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>384</v>
       </c>
@@ -7168,7 +7185,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>387</v>
       </c>
@@ -7179,7 +7196,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>390</v>
       </c>
@@ -7190,7 +7207,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>393</v>
       </c>
@@ -7201,7 +7218,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>396</v>
       </c>
@@ -7212,7 +7229,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>399</v>
       </c>
@@ -7223,7 +7240,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>402</v>
       </c>
@@ -7234,7 +7251,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>405</v>
       </c>
@@ -7245,7 +7262,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>408</v>
       </c>
@@ -7256,7 +7273,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>411</v>
       </c>
@@ -7276,7 +7293,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>416</v>
       </c>
@@ -7296,7 +7313,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>420</v>
       </c>
@@ -7316,7 +7333,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>424</v>
       </c>
@@ -7345,7 +7362,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>432</v>
       </c>
@@ -7374,7 +7391,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>434</v>
       </c>
@@ -7394,7 +7411,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>439</v>
       </c>
@@ -7414,7 +7431,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>444</v>
       </c>
@@ -7434,7 +7451,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>449</v>
       </c>
@@ -7451,7 +7468,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>453</v>
       </c>
@@ -7462,7 +7479,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>456</v>
       </c>
@@ -7473,7 +7490,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>459</v>
       </c>
@@ -7493,7 +7510,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>464</v>
       </c>
@@ -7513,7 +7530,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>469</v>
       </c>
@@ -7539,7 +7556,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>476</v>
       </c>
@@ -7550,7 +7567,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>479</v>
       </c>
@@ -7561,7 +7578,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>482</v>
       </c>
@@ -7572,7 +7589,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>485</v>
       </c>
@@ -7583,7 +7600,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>488</v>
       </c>
@@ -7594,7 +7611,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>491</v>
       </c>
@@ -7605,7 +7622,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>494</v>
       </c>
@@ -7616,7 +7633,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>497</v>
       </c>
@@ -7627,7 +7644,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>500</v>
       </c>
@@ -7638,7 +7655,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>503</v>
       </c>
@@ -7649,7 +7666,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>506</v>
       </c>
@@ -7660,7 +7677,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>509</v>
       </c>
@@ -7671,7 +7688,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>512</v>
       </c>
@@ -7682,7 +7699,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>515</v>
       </c>
@@ -7693,7 +7710,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>518</v>
       </c>
@@ -7704,7 +7721,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>521</v>
       </c>
@@ -7715,7 +7732,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>524</v>
       </c>
@@ -7726,7 +7743,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>527</v>
       </c>
@@ -7737,7 +7754,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>530</v>
       </c>
@@ -7748,7 +7765,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>533</v>
       </c>
@@ -7759,7 +7776,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>536</v>
       </c>
@@ -7770,7 +7787,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>539</v>
       </c>
@@ -7781,7 +7798,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>542</v>
       </c>
@@ -7792,7 +7809,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>545</v>
       </c>
@@ -7803,7 +7820,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>548</v>
       </c>
@@ -7814,7 +7831,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>551</v>
       </c>
@@ -7825,7 +7842,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
         <v>554</v>
       </c>
@@ -7836,7 +7853,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
         <v>557</v>
       </c>
@@ -7847,7 +7864,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
         <v>560</v>
       </c>
@@ -7858,7 +7875,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
         <v>563</v>
       </c>
@@ -7869,7 +7886,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
         <v>566</v>
       </c>
@@ -7880,7 +7897,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A218" t="s">
         <v>569</v>
       </c>
@@ -7891,7 +7908,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A219" t="s">
         <v>572</v>
       </c>
@@ -7902,7 +7919,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A220" t="s">
         <v>575</v>
       </c>
@@ -7913,7 +7930,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A221" t="s">
         <v>578</v>
       </c>
@@ -7924,7 +7941,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A222" t="s">
         <v>581</v>
       </c>
@@ -7935,7 +7952,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A223" t="s">
         <v>584</v>
       </c>
@@ -7946,7 +7963,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A224" t="s">
         <v>587</v>
       </c>
@@ -7957,7 +7974,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A225" t="s">
         <v>590</v>
       </c>
@@ -7968,7 +7985,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A226" t="s">
         <v>593</v>
       </c>
@@ -7979,7 +7996,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A227" t="s">
         <v>596</v>
       </c>
@@ -7990,7 +8007,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A228" t="s">
         <v>599</v>
       </c>
@@ -8001,7 +8018,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A229" t="s">
         <v>602</v>
       </c>
@@ -8012,7 +8029,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
         <v>605</v>
       </c>
@@ -8023,7 +8040,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A231" t="s">
         <v>608</v>
       </c>
@@ -8034,7 +8051,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
         <v>611</v>
       </c>
@@ -8045,7 +8062,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A233" t="s">
         <v>614</v>
       </c>
@@ -8056,7 +8073,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A234" t="s">
         <v>617</v>
       </c>
@@ -8067,7 +8084,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A235" t="s">
         <v>620</v>
       </c>
@@ -8078,7 +8095,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A236" t="s">
         <v>623</v>
       </c>
@@ -8089,7 +8106,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A237" t="s">
         <v>626</v>
       </c>
@@ -8100,7 +8117,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A238" t="s">
         <v>629</v>
       </c>
@@ -8111,7 +8128,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A239" t="s">
         <v>632</v>
       </c>
@@ -8122,7 +8139,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A240" t="s">
         <v>635</v>
       </c>
@@ -8133,7 +8150,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A241" t="s">
         <v>638</v>
       </c>
@@ -8144,7 +8161,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A242" t="s">
         <v>641</v>
       </c>
@@ -8155,7 +8172,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A243" t="s">
         <v>644</v>
       </c>
@@ -8166,7 +8183,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A244" t="s">
         <v>647</v>
       </c>
@@ -8177,7 +8194,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A245" t="s">
         <v>650</v>
       </c>
@@ -8188,7 +8205,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A246" t="s">
         <v>653</v>
       </c>
@@ -8199,7 +8216,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A247" t="s">
         <v>656</v>
       </c>
@@ -8210,7 +8227,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A248" t="s">
         <v>659</v>
       </c>
@@ -8221,7 +8238,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A249" t="s">
         <v>662</v>
       </c>
@@ -8232,7 +8249,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A250" t="s">
         <v>665</v>
       </c>
@@ -8243,7 +8260,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A251" t="s">
         <v>668</v>
       </c>
@@ -8254,7 +8271,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A252" t="s">
         <v>671</v>
       </c>
@@ -8265,7 +8282,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A253" t="s">
         <v>674</v>
       </c>
@@ -8276,7 +8293,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A254" t="s">
         <v>677</v>
       </c>
@@ -8308,7 +8325,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A255" t="s">
         <v>686</v>
       </c>
@@ -8340,7 +8357,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A256" t="s">
         <v>694</v>
       </c>
@@ -8366,7 +8383,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A257" t="s">
         <v>701</v>
       </c>
@@ -8392,7 +8409,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A258" t="s">
         <v>708</v>
       </c>
@@ -8412,7 +8429,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A259" t="s">
         <v>713</v>
       </c>
@@ -8432,7 +8449,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A260" t="s">
         <v>718</v>
       </c>
@@ -8464,7 +8481,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A261" t="s">
         <v>725</v>
       </c>
@@ -8487,7 +8504,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A262" t="s">
         <v>731</v>
       </c>
@@ -8510,7 +8527,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A263" t="s">
         <v>736</v>
       </c>
@@ -8530,7 +8547,7 @@
         <v>1880</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A264" t="s">
         <v>741</v>
       </c>
@@ -8562,7 +8579,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A265" t="s">
         <v>750</v>
       </c>
@@ -8594,7 +8611,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A266" t="s">
         <v>758</v>
       </c>
@@ -8617,7 +8634,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A267" t="s">
         <v>763</v>
       </c>
@@ -8646,7 +8663,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A268" t="s">
         <v>771</v>
       </c>
@@ -8663,7 +8680,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A269" t="s">
         <v>776</v>
       </c>
@@ -8686,7 +8703,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A270" t="s">
         <v>782</v>
       </c>
@@ -8709,7 +8726,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A271" t="s">
         <v>787</v>
       </c>
@@ -8729,7 +8746,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A272" t="s">
         <v>792</v>
       </c>
@@ -8755,7 +8772,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A273" t="s">
         <v>799</v>
       </c>
@@ -8787,7 +8804,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A274" t="s">
         <v>807</v>
       </c>
@@ -8819,7 +8836,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A275" t="s">
         <v>815</v>
       </c>
@@ -8851,7 +8868,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A276" t="s">
         <v>824</v>
       </c>
@@ -8883,7 +8900,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A277" t="s">
         <v>831</v>
       </c>
@@ -8914,6 +8931,528 @@
       <c r="J277" t="s">
         <v>837</v>
       </c>
+    </row>
+    <row r="278" spans="1:500" x14ac:dyDescent="0.45">
+      <c r="A278" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="B278" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="C278" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="D278" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="E278" s="2" t="s">
+        <v>811</v>
+      </c>
+      <c r="F278" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="G278" s="2">
+        <v>2021</v>
+      </c>
+      <c r="H278" s="2">
+        <v>7</v>
+      </c>
+      <c r="I278" s="2">
+        <v>1</v>
+      </c>
+      <c r="J278" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="K278" s="2"/>
+      <c r="L278" s="2"/>
+      <c r="M278" s="2"/>
+      <c r="N278" s="2"/>
+      <c r="O278" s="2"/>
+      <c r="P278" s="2"/>
+      <c r="Q278" s="2"/>
+      <c r="R278" s="2"/>
+      <c r="S278" s="2"/>
+      <c r="T278" s="2"/>
+      <c r="U278" s="2"/>
+      <c r="V278" s="2"/>
+      <c r="W278" s="2"/>
+      <c r="X278" s="2"/>
+      <c r="Y278" s="2"/>
+      <c r="Z278" s="2"/>
+      <c r="AA278" s="2"/>
+      <c r="AB278" s="2"/>
+      <c r="AC278" s="2"/>
+      <c r="AD278" s="2"/>
+      <c r="AE278" s="2"/>
+      <c r="AF278" s="2"/>
+      <c r="AG278" s="2"/>
+      <c r="AH278" s="2"/>
+      <c r="AI278" s="2"/>
+      <c r="AJ278" s="2"/>
+      <c r="AK278" s="2"/>
+      <c r="AL278" s="2"/>
+      <c r="AM278" s="2"/>
+      <c r="AN278" s="2"/>
+      <c r="AO278" s="2"/>
+      <c r="AP278" s="2"/>
+      <c r="AQ278" s="2"/>
+      <c r="AR278" s="2"/>
+      <c r="AS278" s="2"/>
+      <c r="AT278" s="2"/>
+      <c r="AU278" s="2"/>
+      <c r="AV278" s="2"/>
+      <c r="AW278" s="2"/>
+      <c r="AX278" s="2"/>
+      <c r="AY278" s="2"/>
+      <c r="AZ278" s="2"/>
+      <c r="BA278" s="2"/>
+      <c r="BB278" s="2"/>
+      <c r="BC278" s="2"/>
+      <c r="BD278" s="2"/>
+      <c r="BE278" s="2"/>
+      <c r="BF278" s="2"/>
+      <c r="BG278" s="2"/>
+      <c r="BH278" s="2"/>
+      <c r="BI278" s="2"/>
+      <c r="BJ278" s="2"/>
+      <c r="BK278" s="2"/>
+      <c r="BL278" s="2"/>
+      <c r="BM278" s="2"/>
+      <c r="BN278" s="2"/>
+      <c r="BO278" s="2"/>
+      <c r="BP278" s="2"/>
+      <c r="BQ278" s="2"/>
+      <c r="BR278" s="2"/>
+      <c r="BS278" s="2"/>
+      <c r="BT278" s="2"/>
+      <c r="BU278" s="2"/>
+      <c r="BV278" s="2"/>
+      <c r="BW278" s="2"/>
+      <c r="BX278" s="2"/>
+      <c r="BY278" s="2"/>
+      <c r="BZ278" s="2"/>
+      <c r="CA278" s="2"/>
+      <c r="CB278" s="2"/>
+      <c r="CC278" s="2"/>
+      <c r="CD278" s="2"/>
+      <c r="CE278" s="2"/>
+      <c r="CF278" s="2"/>
+      <c r="CG278" s="2"/>
+      <c r="CH278" s="2"/>
+      <c r="CI278" s="2"/>
+      <c r="CJ278" s="2"/>
+      <c r="CK278" s="2"/>
+      <c r="CL278" s="2"/>
+      <c r="CM278" s="2"/>
+      <c r="CN278" s="2"/>
+      <c r="CO278" s="2"/>
+      <c r="CP278" s="2"/>
+      <c r="CQ278" s="2"/>
+      <c r="CR278" s="2"/>
+      <c r="CS278" s="2"/>
+      <c r="CT278" s="2"/>
+      <c r="CU278" s="2"/>
+      <c r="CV278" s="2"/>
+      <c r="CW278" s="2"/>
+      <c r="CX278" s="2"/>
+      <c r="CY278" s="2"/>
+      <c r="CZ278" s="2"/>
+      <c r="DA278" s="2"/>
+      <c r="DB278" s="2"/>
+      <c r="DC278" s="2"/>
+      <c r="DD278" s="2"/>
+      <c r="DE278" s="2"/>
+      <c r="DF278" s="2"/>
+      <c r="DG278" s="2"/>
+      <c r="DH278" s="2"/>
+      <c r="DI278" s="2"/>
+      <c r="DJ278" s="2"/>
+      <c r="DK278" s="2"/>
+      <c r="DL278" s="2"/>
+      <c r="DM278" s="2"/>
+      <c r="DN278" s="2"/>
+      <c r="DO278" s="2"/>
+      <c r="DP278" s="2"/>
+      <c r="DQ278" s="2"/>
+      <c r="DR278" s="2"/>
+      <c r="DS278" s="2"/>
+      <c r="DT278" s="2"/>
+      <c r="DU278" s="2"/>
+      <c r="DV278" s="2"/>
+      <c r="DW278" s="2"/>
+      <c r="DX278" s="2"/>
+      <c r="DY278" s="2"/>
+      <c r="DZ278" s="2"/>
+      <c r="EA278" s="2"/>
+      <c r="EB278" s="2"/>
+      <c r="EC278" s="2"/>
+      <c r="ED278" s="2"/>
+      <c r="EE278" s="2"/>
+      <c r="EF278" s="2"/>
+      <c r="EG278" s="2"/>
+      <c r="EH278" s="2"/>
+      <c r="EI278" s="2"/>
+      <c r="EJ278" s="2"/>
+      <c r="EK278" s="2"/>
+      <c r="EL278" s="2"/>
+      <c r="EM278" s="2"/>
+      <c r="EN278" s="2"/>
+      <c r="EO278" s="2"/>
+      <c r="EP278" s="2"/>
+      <c r="EQ278" s="2"/>
+      <c r="ER278" s="2"/>
+      <c r="ES278" s="2"/>
+      <c r="ET278" s="2"/>
+      <c r="EU278" s="2"/>
+      <c r="EV278" s="2"/>
+      <c r="EW278" s="2"/>
+      <c r="EX278" s="2"/>
+      <c r="EY278" s="2"/>
+      <c r="EZ278" s="2"/>
+      <c r="FA278" s="2"/>
+      <c r="FB278" s="2"/>
+      <c r="FC278" s="2"/>
+      <c r="FD278" s="2"/>
+      <c r="FE278" s="2"/>
+      <c r="FF278" s="2"/>
+      <c r="FG278" s="2"/>
+      <c r="FH278" s="2"/>
+      <c r="FI278" s="2"/>
+      <c r="FJ278" s="2"/>
+      <c r="FK278" s="2"/>
+      <c r="FL278" s="2"/>
+      <c r="FM278" s="2"/>
+      <c r="FN278" s="2"/>
+      <c r="FO278" s="2"/>
+      <c r="FP278" s="2"/>
+      <c r="FQ278" s="2"/>
+      <c r="FR278" s="2"/>
+      <c r="FS278" s="2"/>
+      <c r="FT278" s="2"/>
+      <c r="FU278" s="2"/>
+      <c r="FV278" s="2"/>
+      <c r="FW278" s="2"/>
+      <c r="FX278" s="2"/>
+      <c r="FY278" s="2"/>
+      <c r="FZ278" s="2"/>
+      <c r="GA278" s="2"/>
+      <c r="GB278" s="2"/>
+      <c r="GC278" s="2"/>
+      <c r="GD278" s="2"/>
+      <c r="GE278" s="2"/>
+      <c r="GF278" s="2"/>
+      <c r="GG278" s="2"/>
+      <c r="GH278" s="2"/>
+      <c r="GI278" s="2"/>
+      <c r="GJ278" s="2"/>
+      <c r="GK278" s="2"/>
+      <c r="GL278" s="2"/>
+      <c r="GM278" s="2"/>
+      <c r="GN278" s="2"/>
+      <c r="GO278" s="2"/>
+      <c r="GP278" s="2"/>
+      <c r="GQ278" s="2"/>
+      <c r="GR278" s="2"/>
+      <c r="GS278" s="2"/>
+      <c r="GT278" s="2"/>
+      <c r="GU278" s="2"/>
+      <c r="GV278" s="2"/>
+      <c r="GW278" s="2"/>
+      <c r="GX278" s="2"/>
+      <c r="GY278" s="2"/>
+      <c r="GZ278" s="2"/>
+      <c r="HA278" s="2"/>
+      <c r="HB278" s="2"/>
+      <c r="HC278" s="2"/>
+      <c r="HD278" s="2"/>
+      <c r="HE278" s="2"/>
+      <c r="HF278" s="2"/>
+      <c r="HG278" s="2"/>
+      <c r="HH278" s="2"/>
+      <c r="HI278" s="2"/>
+      <c r="HJ278" s="2"/>
+      <c r="HK278" s="2"/>
+      <c r="HL278" s="2"/>
+      <c r="HM278" s="2"/>
+      <c r="HN278" s="2"/>
+      <c r="HO278" s="2"/>
+      <c r="HP278" s="2"/>
+      <c r="HQ278" s="2"/>
+      <c r="HR278" s="2"/>
+      <c r="HS278" s="2"/>
+      <c r="HT278" s="2"/>
+      <c r="HU278" s="2"/>
+      <c r="HV278" s="2"/>
+      <c r="HW278" s="2"/>
+      <c r="HX278" s="2"/>
+      <c r="HY278" s="2"/>
+      <c r="HZ278" s="2"/>
+      <c r="IA278" s="2"/>
+      <c r="IB278" s="2"/>
+      <c r="IC278" s="2"/>
+      <c r="ID278" s="2"/>
+      <c r="IE278" s="2"/>
+      <c r="IF278" s="2"/>
+      <c r="IG278" s="2"/>
+      <c r="IH278" s="2"/>
+      <c r="II278" s="2"/>
+      <c r="IJ278" s="2"/>
+      <c r="IK278" s="2"/>
+      <c r="IL278" s="2"/>
+      <c r="IM278" s="2"/>
+      <c r="IN278" s="2"/>
+      <c r="IO278" s="2"/>
+      <c r="IP278" s="2"/>
+      <c r="IQ278" s="2"/>
+      <c r="IR278" s="2"/>
+      <c r="IS278" s="2"/>
+      <c r="IT278" s="2"/>
+      <c r="IU278" s="2"/>
+      <c r="IV278" s="2"/>
+      <c r="IW278" s="2"/>
+      <c r="IX278" s="2"/>
+      <c r="IY278" s="2"/>
+      <c r="IZ278" s="2"/>
+      <c r="JA278" s="2"/>
+      <c r="JB278" s="2"/>
+      <c r="JC278" s="2"/>
+      <c r="JD278" s="2"/>
+      <c r="JE278" s="2"/>
+      <c r="JF278" s="2"/>
+      <c r="JG278" s="2"/>
+      <c r="JH278" s="2"/>
+      <c r="JI278" s="2"/>
+      <c r="JJ278" s="2"/>
+      <c r="JK278" s="2"/>
+      <c r="JL278" s="2"/>
+      <c r="JM278" s="2"/>
+      <c r="JN278" s="2"/>
+      <c r="JO278" s="2"/>
+      <c r="JP278" s="2"/>
+      <c r="JQ278" s="2"/>
+      <c r="JR278" s="2"/>
+      <c r="JS278" s="2"/>
+      <c r="JT278" s="2"/>
+      <c r="JU278" s="2"/>
+      <c r="JV278" s="2"/>
+      <c r="JW278" s="2"/>
+      <c r="JX278" s="2"/>
+      <c r="JY278" s="2"/>
+      <c r="JZ278" s="2"/>
+      <c r="KA278" s="2"/>
+      <c r="KB278" s="2"/>
+      <c r="KC278" s="2"/>
+      <c r="KD278" s="2"/>
+      <c r="KE278" s="2"/>
+      <c r="KF278" s="2"/>
+      <c r="KG278" s="2"/>
+      <c r="KH278" s="2"/>
+      <c r="KI278" s="2"/>
+      <c r="KJ278" s="2"/>
+      <c r="KK278" s="2"/>
+      <c r="KL278" s="2"/>
+      <c r="KM278" s="2"/>
+      <c r="KN278" s="2"/>
+      <c r="KO278" s="2"/>
+      <c r="KP278" s="2"/>
+      <c r="KQ278" s="2"/>
+      <c r="KR278" s="2"/>
+      <c r="KS278" s="2"/>
+      <c r="KT278" s="2"/>
+      <c r="KU278" s="2"/>
+      <c r="KV278" s="2"/>
+      <c r="KW278" s="2"/>
+      <c r="KX278" s="2"/>
+      <c r="KY278" s="2"/>
+      <c r="KZ278" s="2"/>
+      <c r="LA278" s="2"/>
+      <c r="LB278" s="2"/>
+      <c r="LC278" s="2"/>
+      <c r="LD278" s="2"/>
+      <c r="LE278" s="2"/>
+      <c r="LF278" s="2"/>
+      <c r="LG278" s="2"/>
+      <c r="LH278" s="2"/>
+      <c r="LI278" s="2"/>
+      <c r="LJ278" s="2"/>
+      <c r="LK278" s="2"/>
+      <c r="LL278" s="2"/>
+      <c r="LM278" s="2"/>
+      <c r="LN278" s="2"/>
+      <c r="LO278" s="2"/>
+      <c r="LP278" s="2"/>
+      <c r="LQ278" s="2"/>
+      <c r="LR278" s="2"/>
+      <c r="LS278" s="2"/>
+      <c r="LT278" s="2"/>
+      <c r="LU278" s="2"/>
+      <c r="LV278" s="2"/>
+      <c r="LW278" s="2"/>
+      <c r="LX278" s="2"/>
+      <c r="LY278" s="2"/>
+      <c r="LZ278" s="2"/>
+      <c r="MA278" s="2"/>
+      <c r="MB278" s="2"/>
+      <c r="MC278" s="2"/>
+      <c r="MD278" s="2"/>
+      <c r="ME278" s="2"/>
+      <c r="MF278" s="2"/>
+      <c r="MG278" s="2"/>
+      <c r="MH278" s="2"/>
+      <c r="MI278" s="2"/>
+      <c r="MJ278" s="2"/>
+      <c r="MK278" s="2"/>
+      <c r="ML278" s="2"/>
+      <c r="MM278" s="2"/>
+      <c r="MN278" s="2"/>
+      <c r="MO278" s="2"/>
+      <c r="MP278" s="2"/>
+      <c r="MQ278" s="2"/>
+      <c r="MR278" s="2"/>
+      <c r="MS278" s="2"/>
+      <c r="MT278" s="2"/>
+      <c r="MU278" s="2"/>
+      <c r="MV278" s="2"/>
+      <c r="MW278" s="2"/>
+      <c r="MX278" s="2"/>
+      <c r="MY278" s="2"/>
+      <c r="MZ278" s="2"/>
+      <c r="NA278" s="2"/>
+      <c r="NB278" s="2"/>
+      <c r="NC278" s="2"/>
+      <c r="ND278" s="2"/>
+      <c r="NE278" s="2"/>
+      <c r="NF278" s="2"/>
+      <c r="NG278" s="2"/>
+      <c r="NH278" s="2"/>
+      <c r="NI278" s="2"/>
+      <c r="NJ278" s="2"/>
+      <c r="NK278" s="2"/>
+      <c r="NL278" s="2"/>
+      <c r="NM278" s="2"/>
+      <c r="NN278" s="2"/>
+      <c r="NO278" s="2"/>
+      <c r="NP278" s="2"/>
+      <c r="NQ278" s="2"/>
+      <c r="NR278" s="2"/>
+      <c r="NS278" s="2"/>
+      <c r="NT278" s="2"/>
+      <c r="NU278" s="2"/>
+      <c r="NV278" s="2"/>
+      <c r="NW278" s="2"/>
+      <c r="NX278" s="2"/>
+      <c r="NY278" s="2"/>
+      <c r="NZ278" s="2"/>
+      <c r="OA278" s="2"/>
+      <c r="OB278" s="2"/>
+      <c r="OC278" s="2"/>
+      <c r="OD278" s="2"/>
+      <c r="OE278" s="2"/>
+      <c r="OF278" s="2"/>
+      <c r="OG278" s="2"/>
+      <c r="OH278" s="2"/>
+      <c r="OI278" s="2"/>
+      <c r="OJ278" s="2"/>
+      <c r="OK278" s="2"/>
+      <c r="OL278" s="2"/>
+      <c r="OM278" s="2"/>
+      <c r="ON278" s="2"/>
+      <c r="OO278" s="2"/>
+      <c r="OP278" s="2"/>
+      <c r="OQ278" s="2"/>
+      <c r="OR278" s="2"/>
+      <c r="OS278" s="2"/>
+      <c r="OT278" s="2"/>
+      <c r="OU278" s="2"/>
+      <c r="OV278" s="2"/>
+      <c r="OW278" s="2"/>
+      <c r="OX278" s="2"/>
+      <c r="OY278" s="2"/>
+      <c r="OZ278" s="2"/>
+      <c r="PA278" s="2"/>
+      <c r="PB278" s="2"/>
+      <c r="PC278" s="2"/>
+      <c r="PD278" s="2"/>
+      <c r="PE278" s="2"/>
+      <c r="PF278" s="2"/>
+      <c r="PG278" s="2"/>
+      <c r="PH278" s="2"/>
+      <c r="PI278" s="2"/>
+      <c r="PJ278" s="2"/>
+      <c r="PK278" s="2"/>
+      <c r="PL278" s="2"/>
+      <c r="PM278" s="2"/>
+      <c r="PN278" s="2"/>
+      <c r="PO278" s="2"/>
+      <c r="PP278" s="2"/>
+      <c r="PQ278" s="2"/>
+      <c r="PR278" s="2"/>
+      <c r="PS278" s="2"/>
+      <c r="PT278" s="2"/>
+      <c r="PU278" s="2"/>
+      <c r="PV278" s="2"/>
+      <c r="PW278" s="2"/>
+      <c r="PX278" s="2"/>
+      <c r="PY278" s="2"/>
+      <c r="PZ278" s="2"/>
+      <c r="QA278" s="2"/>
+      <c r="QB278" s="2"/>
+      <c r="QC278" s="2"/>
+      <c r="QD278" s="2"/>
+      <c r="QE278" s="2"/>
+      <c r="QF278" s="2"/>
+      <c r="QG278" s="2"/>
+      <c r="QH278" s="2"/>
+      <c r="QI278" s="2"/>
+      <c r="QJ278" s="2"/>
+      <c r="QK278" s="2"/>
+      <c r="QL278" s="2"/>
+      <c r="QM278" s="2"/>
+      <c r="QN278" s="2"/>
+      <c r="QO278" s="2"/>
+      <c r="QP278" s="2"/>
+      <c r="QQ278" s="2"/>
+      <c r="QR278" s="2"/>
+      <c r="QS278" s="2"/>
+      <c r="QT278" s="2"/>
+      <c r="QU278" s="2"/>
+      <c r="QV278" s="2"/>
+      <c r="QW278" s="2"/>
+      <c r="QX278" s="2"/>
+      <c r="QY278" s="2"/>
+      <c r="QZ278" s="2"/>
+      <c r="RA278" s="2"/>
+      <c r="RB278" s="2"/>
+      <c r="RC278" s="2"/>
+      <c r="RD278" s="2"/>
+      <c r="RE278" s="2"/>
+      <c r="RF278" s="2"/>
+      <c r="RG278" s="2"/>
+      <c r="RH278" s="2"/>
+      <c r="RI278" s="2"/>
+      <c r="RJ278" s="2"/>
+      <c r="RK278" s="2"/>
+      <c r="RL278" s="2"/>
+      <c r="RM278" s="2"/>
+      <c r="RN278" s="2"/>
+      <c r="RO278" s="2"/>
+      <c r="RP278" s="2"/>
+      <c r="RQ278" s="2"/>
+      <c r="RR278" s="2"/>
+      <c r="RS278" s="2"/>
+      <c r="RT278" s="2"/>
+      <c r="RU278" s="2"/>
+      <c r="RV278" s="2"/>
+      <c r="RW278" s="2"/>
+      <c r="RX278" s="2"/>
+      <c r="RY278" s="2"/>
+      <c r="RZ278" s="2"/>
+      <c r="SA278" s="2"/>
+      <c r="SB278" s="2"/>
+      <c r="SC278" s="2"/>
+      <c r="SD278" s="2"/>
+      <c r="SE278" s="2"/>
+      <c r="SF278" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>